<commit_message>
feat: add AI Chef Pro logo badge on all product pages + fix Excel branding
- New LogoBadge component: white rounded card with logo, links to homepage
- Added to hub, 4 landings, and 4 dashboards (9 pages total)
- Fixed missing branding footer in BONUS-02 calendario Excel

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/dl/kit-tareas/BONUS-02-calendario-anual-tareas.xlsx
+++ b/public/dl/kit-tareas/BONUS-02-calendario-anual-tareas.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -64,6 +64,11 @@
     <font>
       <name val="Calibri"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00888888"/>
+      <sz val="8"/>
     </font>
   </fonts>
   <fills count="5">
@@ -118,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -145,6 +150,9 @@
     </xf>
     <xf applyAlignment="1" borderId="1" fillId="4" fontId="7" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="8" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -533,9 +541,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="B5" t="inlineStr"/>
-    </row>
+    <row r="5"/>
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
         <is>
@@ -557,9 +563,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="B9" t="inlineStr"/>
-    </row>
+    <row r="9"/>
     <row r="10">
       <c r="B10" s="2" t="inlineStr">
         <is>
@@ -579,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col customWidth="1" max="1" min="1" width="15"/>
@@ -1094,9 +1098,17 @@
       </c>
       <c r="D27" s="11" t="inlineStr"/>
     </row>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>— Kit de Tareas Recurrentes · AI Chef Pro · aichef.pro —</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A29:D29"/>
   </mergeCells>
   <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
   <pageSetup orientation="landscape"/>

</xml_diff>